<commit_message>
Remove Zhang Yuyan after she dropped the course and refresh the attendance sheet.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/签到表.xlsx
+++ b/签到表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\ZGCA26SEQF-main\ZGCA26SEQF-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E87D0D6-37A9-4093-9ED6-7FE069E4F593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{02807451-AC3A-46C5-965E-DDD532B48883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5280" yWindow="2520" windowWidth="21600" windowHeight="11295" xr2:uid="{E0C87E15-7E41-4125-B0AA-4472BFD38BAD}"/>
+    <workbookView xWindow="5280" yWindow="2520" windowWidth="21600" windowHeight="11295" xr2:uid="{9BBFB3FC-E601-49D9-9CDD-4D85C8A81870}"/>
   </bookViews>
   <sheets>
     <sheet name="签到表" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>序号</t>
   </si>
@@ -123,9 +123,6 @@
     <t>严从营</t>
   </si>
   <si>
-    <t>张语嫣</t>
-  </si>
-  <si>
     <t>胡家威</t>
   </si>
   <si>
@@ -168,11 +165,10 @@
     <t>日期：________年____月____日</t>
   </si>
   <si>
+    <t>应到 40 人</t>
+  </si>
+  <si>
     <t>实到 ______ 人</t>
-  </si>
-  <si>
-    <t>应到     人</t>
-    <phoneticPr fontId="20" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -798,12 +794,15 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -811,14 +810,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1194,8 +1187,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FECC6DC5-F0EF-46A7-B04C-FB40BE18549C}">
-  <dimension ref="A1:D44"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95A798D3-9ACF-4154-9A01-5A55ED2482AF}">
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.625" customWidth="1"/>
@@ -1205,530 +1198,518 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="3">
+      <c r="A4" s="4">
         <v>1</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="4">
         <v>260301009</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3"/>
+      <c r="D4" s="4"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="3">
+      <c r="A5" s="4">
         <v>2</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="4">
         <v>260303001</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3"/>
+      <c r="D5" s="4"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="3">
+      <c r="A6" s="4">
         <v>3</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="4">
         <v>260303004</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="4"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="3">
+      <c r="A7" s="4">
         <v>4</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="4">
         <v>260403008</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="3"/>
+      <c r="D7" s="4"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
+      <c r="A8" s="4">
         <v>5</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="4">
         <v>260502016</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="3"/>
+      <c r="D8" s="4"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
+      <c r="A9" s="4">
         <v>6</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="4">
         <v>260601061</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="3">
+      <c r="A10" s="4">
         <v>7</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="4">
         <v>260603023</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="3"/>
+      <c r="D10" s="4"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="3">
+      <c r="A11" s="4">
         <v>8</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="4">
         <v>260802035</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="3"/>
+      <c r="D11" s="4"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="3">
+      <c r="A12" s="4">
         <v>9</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="4">
         <v>260802036</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="3"/>
+      <c r="D12" s="4"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="3">
+      <c r="A13" s="4">
         <v>10</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="4">
         <v>260802037</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="3"/>
+      <c r="D13" s="4"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="3">
+      <c r="A14" s="4">
         <v>11</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="4">
         <v>260802040</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D14" s="3"/>
+      <c r="D14" s="4"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="3">
+      <c r="A15" s="4">
         <v>12</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="4">
         <v>260901039</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="3"/>
+      <c r="D15" s="4"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="3">
+      <c r="A16" s="4">
         <v>13</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="4">
         <v>260901042</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="3"/>
+      <c r="D16" s="4"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="3">
+      <c r="A17" s="4">
         <v>14</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="4">
         <v>260901046</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="3"/>
+      <c r="D17" s="4"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="3">
+      <c r="A18" s="4">
         <v>15</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="4">
         <v>260902020</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D18" s="3"/>
+      <c r="D18" s="4"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="3">
+      <c r="A19" s="4">
         <v>16</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="4">
         <v>260902021</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D19" s="3"/>
+      <c r="D19" s="4"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="3">
+      <c r="A20" s="4">
         <v>17</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="4">
         <v>260902023</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="3"/>
+      <c r="D20" s="4"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="3">
+      <c r="A21" s="4">
         <v>18</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="4">
         <v>260902024</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D21" s="3"/>
+      <c r="D21" s="4"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="3">
+      <c r="A22" s="4">
         <v>19</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="4">
         <v>261101073</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D22" s="3"/>
+      <c r="D22" s="4"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="3">
+      <c r="A23" s="4">
         <v>20</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="4">
         <v>261101076</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D23" s="3"/>
+      <c r="D23" s="4"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="3">
+      <c r="A24" s="4">
         <v>21</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="4">
         <v>261102054</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D24" s="3"/>
+      <c r="D24" s="4"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="3">
+      <c r="A25" s="4">
         <v>22</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B25" s="4">
         <v>261102057</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D25" s="3"/>
+      <c r="D25" s="4"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="3">
+      <c r="A26" s="4">
         <v>23</v>
       </c>
-      <c r="B26" s="2">
+      <c r="B26" s="4">
         <v>261301058</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="3"/>
+      <c r="D26" s="4"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="3">
+      <c r="A27" s="4">
         <v>24</v>
       </c>
-      <c r="B27" s="2">
+      <c r="B27" s="4">
         <v>261501099</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D27" s="3"/>
+      <c r="D27" s="4"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="3">
+      <c r="A28" s="4">
         <v>25</v>
       </c>
-      <c r="B28" s="2">
+      <c r="B28" s="4">
         <v>261601103</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="3"/>
+      <c r="D28" s="4"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="3">
+      <c r="A29" s="4">
         <v>26</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29" s="4">
         <v>261601104</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D29" s="3"/>
+      <c r="D29" s="4"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="3">
+      <c r="A30" s="4">
         <v>27</v>
       </c>
-      <c r="B30" s="2">
+      <c r="B30" s="4">
         <v>261601108</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D30" s="3"/>
+      <c r="D30" s="4"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="3">
+      <c r="A31" s="4">
         <v>28</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31" s="4">
         <v>261601110</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D31" s="3"/>
+      <c r="D31" s="4"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="3">
+      <c r="A32" s="4">
         <v>29</v>
       </c>
-      <c r="B32" s="2">
-        <v>261603052</v>
-      </c>
-      <c r="C32" s="2" t="s">
+      <c r="B32" s="4">
+        <v>261702048</v>
+      </c>
+      <c r="C32" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="3"/>
+      <c r="D32" s="4"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="3">
+      <c r="A33" s="4">
         <v>30</v>
       </c>
-      <c r="B33" s="2">
-        <v>261702048</v>
-      </c>
-      <c r="C33" s="2" t="s">
+      <c r="B33" s="4">
+        <v>261703024</v>
+      </c>
+      <c r="C33" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D33" s="3"/>
+      <c r="D33" s="4"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="3">
+      <c r="A34" s="4">
         <v>31</v>
       </c>
-      <c r="B34" s="2">
-        <v>261703024</v>
-      </c>
-      <c r="C34" s="2" t="s">
+      <c r="B34" s="4">
+        <v>262002079</v>
+      </c>
+      <c r="C34" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D34" s="3"/>
+      <c r="D34" s="4"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="3">
+      <c r="A35" s="4">
         <v>32</v>
       </c>
-      <c r="B35" s="2">
-        <v>262002079</v>
-      </c>
-      <c r="C35" s="2" t="s">
+      <c r="B35" s="4">
+        <v>262301119</v>
+      </c>
+      <c r="C35" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D35" s="3"/>
+      <c r="D35" s="4"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="3">
+      <c r="A36" s="4">
         <v>33</v>
       </c>
-      <c r="B36" s="2">
-        <v>262301119</v>
-      </c>
-      <c r="C36" s="2" t="s">
+      <c r="B36" s="4">
+        <v>262301126</v>
+      </c>
+      <c r="C36" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D36" s="3"/>
+      <c r="D36" s="4"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="3">
+      <c r="A37" s="4">
         <v>34</v>
       </c>
-      <c r="B37" s="2">
-        <v>262301126</v>
-      </c>
-      <c r="C37" s="2" t="s">
+      <c r="B37" s="4">
+        <v>262301140</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D37" s="3"/>
+      <c r="D37" s="4"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="3">
+      <c r="A38" s="4">
         <v>35</v>
       </c>
-      <c r="B38" s="2">
-        <v>262301140</v>
-      </c>
-      <c r="C38" s="2" t="s">
+      <c r="B38" s="4">
+        <v>262301142</v>
+      </c>
+      <c r="C38" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D38" s="3"/>
+      <c r="D38" s="4"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="3">
+      <c r="A39" s="4">
         <v>36</v>
       </c>
-      <c r="B39" s="2">
-        <v>262301142</v>
-      </c>
-      <c r="C39" s="2" t="s">
+      <c r="B39" s="4">
+        <v>262501155</v>
+      </c>
+      <c r="C39" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D39" s="3"/>
+      <c r="D39" s="4"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="3">
+      <c r="A40" s="4">
         <v>37</v>
       </c>
-      <c r="B40" s="2">
-        <v>262501155</v>
-      </c>
-      <c r="C40" s="2" t="s">
+      <c r="B40" s="4">
+        <v>262502078</v>
+      </c>
+      <c r="C40" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D40" s="3"/>
+      <c r="D40" s="4"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="3">
+      <c r="A41" s="4">
         <v>38</v>
       </c>
-      <c r="B41" s="2">
-        <v>262502078</v>
-      </c>
-      <c r="C41" s="2" t="s">
+      <c r="B41" s="4">
+        <v>262703034</v>
+      </c>
+      <c r="C41" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D41" s="3"/>
+      <c r="D41" s="4"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="3">
+      <c r="A42" s="4">
         <v>39</v>
       </c>
-      <c r="B42" s="2">
-        <v>262703034</v>
-      </c>
-      <c r="C42" s="2" t="s">
+      <c r="B42" s="4">
+        <v>262802049</v>
+      </c>
+      <c r="C42" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D42" s="3"/>
+      <c r="D42" s="4"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="3">
+      <c r="A43" s="4">
         <v>40</v>
       </c>
-      <c r="B43" s="2">
-        <v>262802049</v>
-      </c>
-      <c r="C43" s="2" t="s">
+      <c r="B43" s="4">
+        <v>262803026</v>
+      </c>
+      <c r="C43" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D43" s="3"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="3">
-        <v>41</v>
-      </c>
-      <c r="B44" s="2">
-        <v>262803026</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D44" s="3"/>
+      <c r="D43" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Remove 11 dropped students and record Lin Yimeng homework 1 as 5.8.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/签到表.xlsx
+++ b/签到表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\ZGCA26SEQF-main\ZGCA26SEQF-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{02807451-AC3A-46C5-965E-DDD532B48883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E24D4245-2B22-46F4-ADE9-F4ABAC8098A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5280" yWindow="2520" windowWidth="21600" windowHeight="11295" xr2:uid="{9BBFB3FC-E601-49D9-9CDD-4D85C8A81870}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B337DFD7-0866-440A-8C35-ECF1B888A541}"/>
   </bookViews>
   <sheets>
     <sheet name="签到表" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>序号</t>
   </si>
@@ -63,12 +63,6 @@
     <t>苏慧康</t>
   </si>
   <si>
-    <t>刘子豪</t>
-  </si>
-  <si>
-    <t>刘挚</t>
-  </si>
-  <si>
     <t>林沂蒙</t>
   </si>
   <si>
@@ -78,18 +72,9 @@
     <t>贾适萌</t>
   </si>
   <si>
-    <t>王庆松</t>
-  </si>
-  <si>
     <t>陈智良</t>
   </si>
   <si>
-    <t>景超</t>
-  </si>
-  <si>
-    <t>李铭鑫</t>
-  </si>
-  <si>
     <t>邵家一</t>
   </si>
   <si>
@@ -105,21 +90,9 @@
     <t>曹祥旭</t>
   </si>
   <si>
-    <t>马思晟</t>
-  </si>
-  <si>
-    <t>马明娇</t>
-  </si>
-  <si>
-    <t>吴铭威</t>
-  </si>
-  <si>
     <t>张哲荣</t>
   </si>
   <si>
-    <t>祁川</t>
-  </si>
-  <si>
     <t>严从营</t>
   </si>
   <si>
@@ -138,9 +111,6 @@
     <t>钟芳梽</t>
   </si>
   <si>
-    <t>姚壮</t>
-  </si>
-  <si>
     <t>黄铮舸</t>
   </si>
   <si>
@@ -156,16 +126,13 @@
     <t>王秋雨</t>
   </si>
   <si>
-    <t>孙恒辉</t>
-  </si>
-  <si>
     <t>2609现代软件工程签到表</t>
   </si>
   <si>
     <t>日期：________年____月____日</t>
   </si>
   <si>
-    <t>应到 40 人</t>
+    <t>应到 29 人</t>
   </si>
   <si>
     <t>实到 ______ 人</t>
@@ -1187,8 +1154,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95A798D3-9ACF-4154-9A01-5A55ED2482AF}">
-  <dimension ref="A1:D43"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B692D704-8183-45CC-B0D0-857A4E12DE52}">
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.625" customWidth="1"/>
@@ -1199,7 +1166,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1207,14 +1174,14 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -1332,7 +1299,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="4">
-        <v>260802036</v>
+        <v>260802040</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>12</v>
@@ -1344,7 +1311,7 @@
         <v>10</v>
       </c>
       <c r="B13" s="4">
-        <v>260802037</v>
+        <v>260901039</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>13</v>
@@ -1356,7 +1323,7 @@
         <v>11</v>
       </c>
       <c r="B14" s="4">
-        <v>260802040</v>
+        <v>260901042</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>14</v>
@@ -1368,7 +1335,7 @@
         <v>12</v>
       </c>
       <c r="B15" s="4">
-        <v>260901039</v>
+        <v>260902020</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>15</v>
@@ -1380,7 +1347,7 @@
         <v>13</v>
       </c>
       <c r="B16" s="4">
-        <v>260901042</v>
+        <v>260902024</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>16</v>
@@ -1392,7 +1359,7 @@
         <v>14</v>
       </c>
       <c r="B17" s="4">
-        <v>260901046</v>
+        <v>261101073</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>17</v>
@@ -1404,7 +1371,7 @@
         <v>15</v>
       </c>
       <c r="B18" s="4">
-        <v>260902020</v>
+        <v>261101076</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>18</v>
@@ -1416,7 +1383,7 @@
         <v>16</v>
       </c>
       <c r="B19" s="4">
-        <v>260902021</v>
+        <v>261102054</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>19</v>
@@ -1428,7 +1395,7 @@
         <v>17</v>
       </c>
       <c r="B20" s="4">
-        <v>260902023</v>
+        <v>261102057</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>20</v>
@@ -1440,7 +1407,7 @@
         <v>18</v>
       </c>
       <c r="B21" s="4">
-        <v>260902024</v>
+        <v>261601104</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>21</v>
@@ -1452,7 +1419,7 @@
         <v>19</v>
       </c>
       <c r="B22" s="4">
-        <v>261101073</v>
+        <v>261601110</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>22</v>
@@ -1464,7 +1431,7 @@
         <v>20</v>
       </c>
       <c r="B23" s="4">
-        <v>261101076</v>
+        <v>261702048</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>23</v>
@@ -1476,7 +1443,7 @@
         <v>21</v>
       </c>
       <c r="B24" s="4">
-        <v>261102054</v>
+        <v>261703024</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>24</v>
@@ -1488,7 +1455,7 @@
         <v>22</v>
       </c>
       <c r="B25" s="4">
-        <v>261102057</v>
+        <v>262002079</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>25</v>
@@ -1500,7 +1467,7 @@
         <v>23</v>
       </c>
       <c r="B26" s="4">
-        <v>261301058</v>
+        <v>262301119</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>26</v>
@@ -1512,7 +1479,7 @@
         <v>24</v>
       </c>
       <c r="B27" s="4">
-        <v>261501099</v>
+        <v>262301126</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>27</v>
@@ -1524,7 +1491,7 @@
         <v>25</v>
       </c>
       <c r="B28" s="4">
-        <v>261601103</v>
+        <v>262301142</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>28</v>
@@ -1536,7 +1503,7 @@
         <v>26</v>
       </c>
       <c r="B29" s="4">
-        <v>261601104</v>
+        <v>262501155</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>29</v>
@@ -1548,7 +1515,7 @@
         <v>27</v>
       </c>
       <c r="B30" s="4">
-        <v>261601108</v>
+        <v>262502078</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>30</v>
@@ -1560,7 +1527,7 @@
         <v>28</v>
       </c>
       <c r="B31" s="4">
-        <v>261601110</v>
+        <v>262703034</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>31</v>
@@ -1572,144 +1539,12 @@
         <v>29</v>
       </c>
       <c r="B32" s="4">
-        <v>261702048</v>
+        <v>262802049</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>32</v>
       </c>
       <c r="D32" s="4"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="4">
-        <v>30</v>
-      </c>
-      <c r="B33" s="4">
-        <v>261703024</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D33" s="4"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="4">
-        <v>31</v>
-      </c>
-      <c r="B34" s="4">
-        <v>262002079</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D34" s="4"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="4">
-        <v>32</v>
-      </c>
-      <c r="B35" s="4">
-        <v>262301119</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D35" s="4"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="4">
-        <v>33</v>
-      </c>
-      <c r="B36" s="4">
-        <v>262301126</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D36" s="4"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="4">
-        <v>34</v>
-      </c>
-      <c r="B37" s="4">
-        <v>262301140</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D37" s="4"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="4">
-        <v>35</v>
-      </c>
-      <c r="B38" s="4">
-        <v>262301142</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D38" s="4"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="4">
-        <v>36</v>
-      </c>
-      <c r="B39" s="4">
-        <v>262501155</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D39" s="4"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="4">
-        <v>37</v>
-      </c>
-      <c r="B40" s="4">
-        <v>262502078</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D40" s="4"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="4">
-        <v>38</v>
-      </c>
-      <c r="B41" s="4">
-        <v>262703034</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D41" s="4"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="4">
-        <v>39</v>
-      </c>
-      <c r="B42" s="4">
-        <v>262802049</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D42" s="4"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="4">
-        <v>40</v>
-      </c>
-      <c r="B43" s="4">
-        <v>262803026</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D43" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>